<commit_message>
mejoras de formato condicional
</commit_message>
<xml_diff>
--- a/models/template.xlsx
+++ b/models/template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ernesto Palacios\GIT\pandas-to-excel-automation\templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/474e2f0e930ab59f/01 JEZO/temp_JEZO_borrar/0000 editar imagenes/reportes/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2AE73D08-7C30-41C9-AF28-0691A2EC7845}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="28" documentId="13_ncr:1_{2AE73D08-7C30-41C9-AF28-0691A2EC7845}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{70311EDD-2220-475F-8C6E-C914382C8CB4}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="28560" windowHeight="14775" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="26490" windowHeight="15390" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="LISTAS" sheetId="1" r:id="rId1"/>
@@ -3635,10 +3635,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="3">
-    <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
-    <numFmt numFmtId="165" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
-    <numFmt numFmtId="166" formatCode="dd/mm/yyyy\ h:mm"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
   </numFmts>
   <fonts count="6" x14ac:knownFonts="1">
     <font>
@@ -3792,7 +3790,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -3804,7 +3802,7 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="3" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -3816,7 +3814,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -3826,13 +3824,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="3" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -3845,7 +3843,24 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="65">
+  <dxfs count="236">
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color rgb="FF000000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC00000"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -3904,19 +3919,17 @@
     </dxf>
     <dxf>
       <font>
-        <b/>
-        <i val="0"/>
+        <color theme="1" tint="0.499984740745262"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF000000"/>
       </font>
     </dxf>
     <dxf>
       <font>
         <color theme="3"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1" tint="0.499984740745262"/>
       </font>
     </dxf>
     <dxf>
@@ -3945,6 +3958,1708 @@
     </dxf>
     <dxf>
       <font>
+        <b/>
+        <i val="0"/>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color theme="1" tint="0.34998626667073579"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF99"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1" tint="0.499984740745262"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color rgb="FF000000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC00000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color rgb="FF77933C"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color rgb="FFFFC000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF000000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="3"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFFFFFF"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="1" tint="0.3498947111423078"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color theme="1" tint="0.34998626667073579"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF99"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color rgb="FF000000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC00000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color rgb="FF77933C"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color rgb="FFFFC000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1" tint="0.499984740745262"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF000000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="3"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFFFFFF"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="1" tint="0.3498947111423078"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color theme="1" tint="0.34998626667073579"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF99"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color rgb="FF000000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC00000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color rgb="FF77933C"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color rgb="FFFFC000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1" tint="0.499984740745262"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF000000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="3"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFFFFFF"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="1" tint="0.3498947111423078"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color theme="1" tint="0.34998626667073579"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF99"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color rgb="FF000000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC00000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color rgb="FF77933C"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color rgb="FFFFC000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1" tint="0.499984740745262"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF000000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="3"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFFFFFF"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="1" tint="0.3498947111423078"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color theme="1" tint="0.34998626667073579"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF99"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color rgb="FF000000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC00000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color rgb="FF77933C"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color rgb="FFFFC000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1" tint="0.499984740745262"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF000000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="3"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFFFFFF"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="1" tint="0.3498947111423078"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color theme="1" tint="0.34998626667073579"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF99"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC00000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color rgb="FF77933C"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color rgb="FFFFC000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1" tint="0.499984740745262"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF000000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="3"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFFFFFF"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="1" tint="0.3498947111423078"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color rgb="FF000000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color theme="1" tint="0.34998626667073579"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF99"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC00000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color rgb="FF77933C"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color rgb="FFFFC000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1" tint="0.499984740745262"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF000000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="3"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFFFFFF"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="1" tint="0.3498947111423078"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color rgb="FF000000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color theme="1" tint="0.34998626667073579"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF99"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC00000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color rgb="FF77933C"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color rgb="FFFFC000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1" tint="0.499984740745262"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF000000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="3"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFFFFFF"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="1" tint="0.3498947111423078"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color rgb="FF000000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color theme="1" tint="0.34998626667073579"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF99"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC00000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color rgb="FF77933C"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color rgb="FFFFC000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1" tint="0.499984740745262"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF000000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="3"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFFFFFF"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="1" tint="0.3498947111423078"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color rgb="FF000000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color theme="1" tint="0.34998626667073579"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF99"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color rgb="FF77933C"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color rgb="FFFFC000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC00000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1" tint="0.499984740745262"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF000000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="3"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFFFFFF"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="1" tint="0.3498947111423078"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color rgb="FF000000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color theme="1" tint="0.34998626667073579"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF99"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color rgb="FF77933C"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color rgb="FFFFC000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC00000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1" tint="0.499984740745262"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF000000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="3"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFFFFFF"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="1" tint="0.3498947111423078"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
         <color rgb="FF000000"/>
       </font>
     </dxf>
@@ -4050,19 +5765,17 @@
     </dxf>
     <dxf>
       <font>
-        <b/>
-        <i val="0"/>
+        <color theme="1" tint="0.499984740745262"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF000000"/>
       </font>
     </dxf>
     <dxf>
       <font>
         <color theme="3"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1" tint="0.499984740745262"/>
       </font>
     </dxf>
     <dxf>
@@ -4091,6 +5804,8 @@
     </dxf>
     <dxf>
       <font>
+        <b/>
+        <i val="0"/>
         <color rgb="FF000000"/>
       </font>
     </dxf>
@@ -4196,19 +5911,17 @@
     </dxf>
     <dxf>
       <font>
-        <b/>
-        <i val="0"/>
+        <color theme="1" tint="0.499984740745262"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF000000"/>
       </font>
     </dxf>
     <dxf>
       <font>
         <color theme="3"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1" tint="0.499984740745262"/>
       </font>
     </dxf>
     <dxf>
@@ -4237,162 +5950,8 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF000000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
         <b/>
         <i val="0"/>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color theme="1" tint="0.34998626667073579"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFF99"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FF77933C"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FFFFC000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FF000000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="3"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFFFFFFF"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFFFFFFF"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="1" tint="0.3498947111423078"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
         <color rgb="FF000000"/>
       </font>
     </dxf>
@@ -5469,7 +7028,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>94</v>
+        <v>44</v>
       </c>
       <c r="C4" s="6" t="s">
         <v>95</v>
@@ -5541,7 +7100,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>79</v>
+        <v>44</v>
       </c>
       <c r="C5" s="17" t="s">
         <v>97</v>
@@ -22153,7 +23712,7 @@
         <v>0</v>
       </c>
       <c r="S235" s="4" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="T235" s="4" t="s">
         <v>32</v>
@@ -34933,63 +36492,70 @@
   </sheetData>
   <autoFilter ref="A1:W293" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
   <conditionalFormatting sqref="A1:A1048576 L1:L1048576">
-    <cfRule type="containsText" dxfId="15" priority="9" operator="containsText" text="domingo">
+    <cfRule type="containsText" dxfId="33" priority="10" operator="containsText" text="sábado">
+      <formula>NOT(ISERROR(SEARCH("sábado",A1)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="32" priority="11" operator="containsText" text="domingo">
       <formula>NOT(ISERROR(SEARCH("domingo",A1)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="14" priority="7" operator="containsText" text="sábado">
-      <formula>NOT(ISERROR(SEARCH("sábado",A1)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A1:X1048576">
-    <cfRule type="expression" dxfId="13" priority="5" stopIfTrue="1">
+    <cfRule type="expression" dxfId="31" priority="8">
       <formula>$A1=1</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="12" priority="14" stopIfTrue="1">
+    <cfRule type="expression" dxfId="30" priority="16">
       <formula>$B1="se_labora"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B1:C1048576">
-    <cfRule type="cellIs" dxfId="11" priority="17" operator="equal">
+    <cfRule type="cellIs" dxfId="29" priority="17" operator="equal">
+      <formula>"se_labora"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="28" priority="18">
+      <formula>($B1=" ALUMBRADO")</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="27" priority="20" operator="equal">
       <formula>"MEDIDORES"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="10" priority="15" operator="equal">
-      <formula>"se_labora"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="9" priority="18" operator="equal">
-      <formula>"informativa"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="8" priority="16" operator="equal">
-      <formula>"ALUMBRADO"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="7" priority="4" stopIfTrue="1" operator="equal">
-      <formula>"REDES"</formula>
+    <cfRule type="expression" dxfId="17" priority="19">
+      <formula>OR(B1="informativa", B1=" lunch ", B1="transporte")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C1:C1048576">
-    <cfRule type="expression" dxfId="6" priority="19">
+    <cfRule type="expression" dxfId="26" priority="1">
       <formula>$S1="Si"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D1:D1048576">
-    <cfRule type="containsText" dxfId="5" priority="1" operator="containsText" text="NO PROG">
+    <cfRule type="containsText" dxfId="25" priority="3" operator="containsText" text="NO PROG">
       <formula>NOT(ISERROR(SEARCH("NO PROG",D1)))</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="4" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="24" priority="5" operator="equal">
       <formula>"PROG"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I1:I1048576">
-    <cfRule type="cellIs" dxfId="3" priority="10" operator="equal">
+    <cfRule type="cellIs" dxfId="23" priority="12" operator="equal">
       <formula>"EXPANSION"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="11" operator="equal">
+    <cfRule type="cellIs" dxfId="22" priority="13" operator="equal">
       <formula>"PREDICTIVO"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="12" operator="equal">
+    <cfRule type="cellIs" dxfId="21" priority="14" operator="equal">
       <formula>"PREVENTIVO"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="13" operator="equal">
+    <cfRule type="cellIs" dxfId="20" priority="15" operator="equal">
       <formula>"CORRECTIVO"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="S1:S1048576">
+    <cfRule type="expression" dxfId="19" priority="2">
+      <formula>AND($S1="Si",$R1=0)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B1:B1048576">
+    <cfRule type="expression" dxfId="18" priority="6">
+      <formula>($B1=" REDES")</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Ahora las condiciones se generan desde OpenPyXL para hora_extra_template.
</commit_message>
<xml_diff>
--- a/models/template.xlsx
+++ b/models/template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/474e2f0e930ab59f/01 JEZO/temp_JEZO_borrar/0000 editar imagenes/reportes/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="28" documentId="13_ncr:1_{2AE73D08-7C30-41C9-AF28-0691A2EC7845}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{70311EDD-2220-475F-8C6E-C914382C8CB4}"/>
+  <xr:revisionPtr revIDLastSave="35" documentId="13_ncr:1_{2AE73D08-7C30-41C9-AF28-0691A2EC7845}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5AD97D81-75FE-40E3-943C-53224826A764}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="26490" windowHeight="15390" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15720" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="LISTAS" sheetId="1" r:id="rId1"/>
@@ -3843,175 +3843,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="236">
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FF000000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC00000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FF77933C"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FFFFC000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1" tint="0.499984740745262"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF000000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="3"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFFFFFFF"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="1" tint="0.3498947111423078"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color theme="1" tint="0.34998626667073579"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFF99"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1" tint="0.499984740745262"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FF000000"/>
-      </font>
-    </dxf>
+  <dxfs count="51">
     <dxf>
       <font>
         <color theme="0"/>
@@ -4085,775 +3917,7 @@
     </dxf>
     <dxf>
       <font>
-        <color theme="3"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFFFFFFF"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="1" tint="0.3498947111423078"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color theme="1" tint="0.34998626667073579"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFF99"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FF000000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC00000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FF77933C"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FFFFC000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
         <color theme="1" tint="0.499984740745262"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF000000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="3"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFFFFFFF"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="1" tint="0.3498947111423078"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color theme="1" tint="0.34998626667073579"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFF99"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FF000000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC00000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FF77933C"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FFFFC000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1" tint="0.499984740745262"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF000000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="3"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFFFFFFF"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="1" tint="0.3498947111423078"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color theme="1" tint="0.34998626667073579"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFF99"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FF000000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC00000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FF77933C"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FFFFC000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1" tint="0.499984740745262"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF000000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="3"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFFFFFFF"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="1" tint="0.3498947111423078"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color theme="1" tint="0.34998626667073579"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFF99"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FF000000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC00000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FF77933C"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FFFFC000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1" tint="0.499984740745262"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF000000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="3"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFFFFFFF"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="1" tint="0.3498947111423078"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color theme="1" tint="0.34998626667073579"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFF99"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC00000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FF77933C"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FFFFC000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1" tint="0.499984740745262"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF000000"/>
       </font>
     </dxf>
     <dxf>
@@ -5004,12 +4068,12 @@
     </dxf>
     <dxf>
       <font>
-        <color theme="1" tint="0.499984740745262"/>
+        <color rgb="FF000000"/>
       </font>
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF000000"/>
+        <color theme="1" tint="0.499984740745262"/>
       </font>
     </dxf>
     <dxf>
@@ -5160,763 +4224,12 @@
     </dxf>
     <dxf>
       <font>
-        <color theme="1" tint="0.499984740745262"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
         <color rgb="FF000000"/>
       </font>
     </dxf>
     <dxf>
       <font>
-        <color theme="3"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFFFFFFF"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="1" tint="0.3498947111423078"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FF000000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color theme="1" tint="0.34998626667073579"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFF99"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC00000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FF77933C"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FFFFC000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
         <color theme="1" tint="0.499984740745262"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF000000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="3"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFFFFFFF"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="1" tint="0.3498947111423078"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FF000000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color theme="1" tint="0.34998626667073579"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFF99"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FF77933C"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FFFFC000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC00000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1" tint="0.499984740745262"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF000000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="3"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFFFFFFF"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="1" tint="0.3498947111423078"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FF000000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color theme="1" tint="0.34998626667073579"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFF99"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FF77933C"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FFFFC000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC00000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1" tint="0.499984740745262"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF000000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="3"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFFFFFFF"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="1" tint="0.3498947111423078"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FF000000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color theme="1" tint="0.34998626667073579"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFF99"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FF77933C"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FFFFC000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1" tint="0.499984740745262"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF000000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="3"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFFFFFFF"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="1" tint="0.3498947111423078"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FF000000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color theme="1" tint="0.34998626667073579"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFF99"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FF77933C"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FFFFC000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1" tint="0.499984740745262"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF000000"/>
       </font>
     </dxf>
     <dxf>
@@ -6081,6 +4394,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -7748,7 +6065,7 @@
         <v>7</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>117</v>
+        <v>5</v>
       </c>
       <c r="C14" s="17" t="s">
         <v>1026</v>
@@ -8088,7 +6405,7 @@
         <v>1</v>
       </c>
       <c r="S18" s="4" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="T18" s="4" t="s">
         <v>111</v>
@@ -26520,7 +24837,7 @@
         <v>1</v>
       </c>
       <c r="S274" s="4" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="T274" s="4" t="s">
         <v>87</v>
@@ -36507,55 +34824,55 @@
       <formula>$B1="se_labora"</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="B1:B1048576">
+    <cfRule type="expression" dxfId="29" priority="6">
+      <formula>($B1=" REDES")</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="B1:C1048576">
-    <cfRule type="cellIs" dxfId="29" priority="17" operator="equal">
+    <cfRule type="cellIs" dxfId="28" priority="17" operator="equal">
       <formula>"se_labora"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="28" priority="18">
+    <cfRule type="expression" dxfId="27" priority="18">
       <formula>($B1=" ALUMBRADO")</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="27" priority="20" operator="equal">
+    <cfRule type="expression" dxfId="26" priority="19">
+      <formula>OR(B1="informativa", B1=" lunch ", B1="transporte")</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="25" priority="20" operator="equal">
       <formula>"MEDIDORES"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="17" priority="19">
-      <formula>OR(B1="informativa", B1=" lunch ", B1="transporte")</formula>
-    </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C1:C1048576">
-    <cfRule type="expression" dxfId="26" priority="1">
+  <conditionalFormatting sqref="C1:C1048576 S1:S1048576">
+    <cfRule type="expression" dxfId="24" priority="2">
       <formula>$S1="Si"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D1:D1048576">
-    <cfRule type="containsText" dxfId="25" priority="3" operator="containsText" text="NO PROG">
+    <cfRule type="containsText" dxfId="23" priority="3" operator="containsText" text="NO PROG">
       <formula>NOT(ISERROR(SEARCH("NO PROG",D1)))</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="24" priority="5" operator="equal">
+    <cfRule type="cellIs" dxfId="22" priority="5" operator="equal">
       <formula>"PROG"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I1:I1048576">
-    <cfRule type="cellIs" dxfId="23" priority="12" operator="equal">
+    <cfRule type="cellIs" dxfId="21" priority="12" operator="equal">
       <formula>"EXPANSION"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="22" priority="13" operator="equal">
+    <cfRule type="cellIs" dxfId="20" priority="13" operator="equal">
       <formula>"PREDICTIVO"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="21" priority="14" operator="equal">
+    <cfRule type="cellIs" dxfId="19" priority="14" operator="equal">
       <formula>"PREVENTIVO"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="20" priority="15" operator="equal">
+    <cfRule type="cellIs" dxfId="18" priority="15" operator="equal">
       <formula>"CORRECTIVO"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="S1:S1048576">
-    <cfRule type="expression" dxfId="19" priority="2">
+    <cfRule type="expression" dxfId="17" priority="1">
       <formula>AND($S1="Si",$R1=0)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B1:B1048576">
-    <cfRule type="expression" dxfId="18" priority="6">
-      <formula>($B1=" REDES")</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>